<commit_message>
Update verification flow to 3-selfie approach, add verify-to-unlock messaging, fix age restriction gating
</commit_message>
<xml_diff>
--- a/Nigh_Subscriptions_CurrentThinking.xlsx
+++ b/Nigh_Subscriptions_CurrentThinking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshritzer/Desktop/Nigh old docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F3753D-3870-C347-9785-2C1C316A3A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB3889B-F7E0-E443-B44C-CB85AFB66197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2160" yWindow="2540" windowWidth="29200" windowHeight="18300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,20 @@
     <sheet name="Capability Analysis" sheetId="8" r:id="rId9"/>
     <sheet name="Strategy Summary" sheetId="9" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
Clean up: archive 40+ old prototypes and legacy files, keep only active versions referenced by index.html
</commit_message>
<xml_diff>
--- a/Nigh_Subscriptions_CurrentThinking.xlsx
+++ b/Nigh_Subscriptions_CurrentThinking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshritzer/Desktop/Nigh old docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB3889B-F7E0-E443-B44C-CB85AFB66197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{568D2244-38D1-C94D-B313-86E5D6336229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2160" yWindow="2540" windowWidth="29200" windowHeight="18300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5129" uniqueCount="1461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5128" uniqueCount="1462">
   <si>
     <t>Nigh Host — Current Access / Verification / Subscription Thinking</t>
   </si>
@@ -4435,21 +4435,24 @@
     <t>Verification required</t>
   </si>
   <si>
-    <t>Free</t>
-  </si>
-  <si>
-    <t>Free 
+    <t>3 per week</t>
+  </si>
+  <si>
+    <t>Free drop fee</t>
+  </si>
+  <si>
+    <t>Drops (per week or per day)</t>
+  </si>
+  <si>
+    <t>Pro (or Growth)
 (w/ verified)</t>
   </si>
   <si>
-    <t>Pro
+    <t>Starter (or Free)
 (w/ verified)</t>
   </si>
   <si>
-    <t>3 per week</t>
-  </si>
-  <si>
-    <t>Free drop fee</t>
+    <t>Starter (or Free)</t>
   </si>
 </sst>
 </file>
@@ -9389,13 +9392,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="187" t="s">
-        <v>1456</v>
+        <v>1461</v>
       </c>
       <c r="C5" s="187" t="s">
-        <v>1457</v>
+        <v>1460</v>
       </c>
       <c r="D5" s="187" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="E5" s="140" t="s">
         <v>616</v>
@@ -9456,7 +9459,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="184" t="s">
-        <v>1460</v>
+        <v>1457</v>
       </c>
       <c r="B9" s="142" t="s">
         <v>28</v>
@@ -9485,7 +9488,7 @@
         <v>18</v>
       </c>
       <c r="D10" s="145" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10" s="145" t="s">
         <v>14</v>
@@ -9734,13 +9737,13 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="184" t="s">
-        <v>631</v>
+        <v>1458</v>
       </c>
       <c r="B24" s="182" t="s">
-        <v>1459</v>
+        <v>1456</v>
       </c>
       <c r="C24" s="182" t="s">
-        <v>1459</v>
+        <v>1456</v>
       </c>
       <c r="D24" s="182" t="s">
         <v>1448</v>
@@ -10675,8 +10678,8 @@
       <c r="B73" s="145" t="s">
         <v>780</v>
       </c>
-      <c r="C73" s="145" t="s">
-        <v>888</v>
+      <c r="C73" s="145">
+        <v>3</v>
       </c>
       <c r="D73" s="145">
         <v>7</v>

</xml_diff>